<commit_message>
IN Piura: declarar el alcance de los promedios en la hoja Microcuenca
AVERAGE omite las celdas de texto «Por determinar», de modo que un promedio
calculado sobre un subconjunto de los bloques de la microcuenca se veia
identico a uno completo. Se anade una nota que declara sobre cuantos bloques
se calcula cada promedio y cuantos carecen del dato de origen (MDE para
pendiente y MSAVI; estadistica zonal para NDVI). Afecta a 9 bloques en
pendiente/MSAVI y a 35 en vegetacion alta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aw2xnniBKHWu654Yk7My2q
</commit_message>
<xml_diff>
--- a/in_piura_plantillas/salida/Plantilla_Excel_Bloque_18_IN_Piura.xlsx
+++ b/in_piura_plantillas/salida/Plantilla_Excel_Bloque_18_IN_Piura.xlsx
@@ -2236,7 +2236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2707,31 +2707,39 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="84" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>ALCANCE DE LOS PROMEDIOS. La fila TOTAL / PROMEDIO omite las celdas «Por determinar»: el promedio de VEGETACIÓN ALTA (NDVI 2025) se calcula sobre 9 de los 11 bloques; los 2 bloques restantes carecen de estadística zonal de NDVI. Los totales de ÁREA y % de microcuenca sí comprenden la totalidad de los 11 bloques. No se estima ningún valor ausente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="84" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>LECTURA INTRAMICROCUENCA. El bloque 18 ocupa el puesto 1 de 11 por superficie dentro de la microcuenca C1076-Q9592 (21.54 % de las 481.17 ha preliminares de la microcuenca). Su pendiente promedio (28.70 %, clase «25-50% (Mod. escarpado)») es la 7.ª más baja de 11 y se sitúa por debajo del promedio de la microcuenca (29.39 %). Su MSAVI 2024 (0.6402) es el 1.º de 11 y queda por encima del promedio local (0.5435). Amplitud altitudinal del bloque: 686 m (1218–1904 msnm). El cuadro conserva todos los bloques catalogados en la microcuenca, incluidos los descartados en el tamizaje, para referencia del conjunto. Los bloques sin ficha DT figuran con sus parámetros de gabinete.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>NOTA METODOLÓGICA. Área y MSAVI 2024 proceden del catálogo maestro de bloques V5/V6. El rango altitudinal y la pendiente promedio proceden del reporte de estadística zonal sobre el MDE («Rango de altitud y Pendiente Promedio por Bloques V6»). El porcentaje de «Vegetación alta» procede de la estadística zonal del NDVI mediana 2025 (Sentinel-2). Los totales y promedios se calculan con fórmulas sobre las filas del cuadro.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A23:H23"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>